<commit_message>
feat: land CombatConstantConfig P0-P2, PushMap camera intro, and Mode2 StartBattle layout (v0.82.38)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/通用_常量表_Combat_CombatConstantConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/通用_常量表_Combat_CombatConstantConfig.xlsx
@@ -39,50 +39,50 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="235">
   <si>
     <t>常量键</t>
   </si>
   <si>
+    <t>主键中文翻译</t>
+  </si>
+  <si>
+    <t>数值</t>
+  </si>
+  <si>
+    <t>备注</t>
+  </si>
+  <si>
+    <t>备注中文解释</t>
+  </si>
+  <si>
     <t>主键</t>
   </si>
   <si>
+    <t>展示用中文名；运行时不读</t>
+  </si>
+  <si>
+    <t>float</t>
+  </si>
+  <si>
+    <t>英文备注；运行时不读</t>
+  </si>
+  <si>
+    <t>中文说明；运行时不读</t>
+  </si>
+  <si>
     <t>ConstantKey</t>
   </si>
   <si>
-    <t>主键中文翻译</t>
-  </si>
-  <si>
-    <t>展示用中文名；运行时不读</t>
-  </si>
-  <si>
     <t>ConstantKeyZh</t>
   </si>
   <si>
-    <t>数值</t>
-  </si>
-  <si>
-    <t>float</t>
-  </si>
-  <si>
     <t>Value</t>
   </si>
   <si>
-    <t>备注</t>
-  </si>
-  <si>
-    <t>英文备注；运行时不读</t>
-  </si>
-  <si>
     <t>Comment</t>
   </si>
   <si>
-    <t>备注中文解释</t>
-  </si>
-  <si>
-    <t>中文说明；运行时不读</t>
-  </si>
-  <si>
     <t>CommentZh</t>
   </si>
   <si>
@@ -107,7 +107,7 @@
     <t>AttackSpeed constant term</t>
   </si>
   <si>
-    <t>攻速=本值+AttackSpeedAgiDiv/max(敏捷,1)中的常数项</t>
+    <t>攻速=本值+敏捷相关项中的常数项</t>
   </si>
   <si>
     <t>AttackSpeedAgiDiv</t>
@@ -156,6 +156,594 @@
   </si>
   <si>
     <t>士兵最大生命=ceil(躯体生命+力量×本系数)</t>
+  </si>
+  <si>
+    <t>CameraHeightY</t>
+  </si>
+  <si>
+    <t>镜头高度</t>
+  </si>
+  <si>
+    <t>Top-down camera world Y above map center</t>
+  </si>
+  <si>
+    <t>俯视正交相机相对地图中心的世界Y高度；Dig/Defend/布阵/PushMap共用</t>
+  </si>
+  <si>
+    <t>CameraOrthoSizeMargin</t>
+  </si>
+  <si>
+    <t>地图适配Size余量</t>
+  </si>
+  <si>
+    <t>orthoSize = max(halfExtents) - margin</t>
+  </si>
+  <si>
+    <t>Dig/Defend/布阵：正交Size=地图半幅较大边减去本余量</t>
+  </si>
+  <si>
+    <t>PushMapCameraOrthoSize</t>
+  </si>
+  <si>
+    <t>推图开战默认Size</t>
+  </si>
+  <si>
+    <t>PushMap combat default orthographicSize</t>
+  </si>
+  <si>
+    <t>PushMap开战默认正交Size（异于Defend的地图适配公式）</t>
+  </si>
+  <si>
+    <t>CameraNearClip</t>
+  </si>
+  <si>
+    <t>镜头近裁剪面</t>
+  </si>
+  <si>
+    <t>Camera nearClipPlane</t>
+  </si>
+  <si>
+    <t>正交相机近裁剪面</t>
+  </si>
+  <si>
+    <t>CameraFarClip</t>
+  </si>
+  <si>
+    <t>镜头远裁剪面</t>
+  </si>
+  <si>
+    <t>Camera farClipPlane</t>
+  </si>
+  <si>
+    <t>正交相机远裁剪面</t>
+  </si>
+  <si>
+    <t>CameraFollowDeadzone</t>
+  </si>
+  <si>
+    <t>跟随死区半径</t>
+  </si>
+  <si>
+    <t>PushMap Auto follow deadzone world-XZ</t>
+  </si>
+  <si>
+    <t>PushMap Auto跟随：目标在死区内则镜头XZ不移动</t>
+  </si>
+  <si>
+    <t>CameraFollowSmoothTime</t>
+  </si>
+  <si>
+    <t>跟随平滑时间</t>
+  </si>
+  <si>
+    <t>PushMap Auto SmoothDamp time</t>
+  </si>
+  <si>
+    <t>PushMap Auto跟随：超出死区后XZ SmoothDamp时间（秒）</t>
+  </si>
+  <si>
+    <t>CameraZoomStepPerNotch</t>
+  </si>
+  <si>
+    <t>滚轮缩放步进</t>
+  </si>
+  <si>
+    <t>Scroll wheel orthographicSize step</t>
+  </si>
+  <si>
+    <t>PushMap滚轮每格改变的正交Size</t>
+  </si>
+  <si>
+    <t>CameraOrthoSizeMin</t>
+  </si>
+  <si>
+    <t>正交Size下限</t>
+  </si>
+  <si>
+    <t>Min orthographicSize clamp</t>
+  </si>
+  <si>
+    <t>正交Size下限（含Dig/Defend适配结果钳制与PushMap缩放）</t>
+  </si>
+  <si>
+    <t>CameraOrthoSizeMax</t>
+  </si>
+  <si>
+    <t>正交Size上限</t>
+  </si>
+  <si>
+    <t>Max orthographicSize clamp</t>
+  </si>
+  <si>
+    <t>PushMap滚轮缩放上限</t>
+  </si>
+  <si>
+    <t>CameraDragThresholdPixels</t>
+  </si>
+  <si>
+    <t>拖拽启动像素阈值</t>
+  </si>
+  <si>
+    <t>LMB drag arm threshold in screen px</t>
+  </si>
+  <si>
+    <t>PushMap手动拖镜头：累计位移超过本像素才开始平移</t>
+  </si>
+  <si>
+    <t>PushMapCameraIntroSpeed</t>
+  </si>
+  <si>
+    <t>推图镜头预览速度</t>
+  </si>
+  <si>
+    <t>PushMap StartBattle Intro rail speed world-XZ units/sec</t>
+  </si>
+  <si>
+    <t>PushMap开战镜头预览沿CameraFollowPath的世界XZ恒速（单位/秒）</t>
+  </si>
+  <si>
+    <t>PushMapCameraIntroWaypointDwellSeconds</t>
+  </si>
+  <si>
+    <t>推图镜头预览路点停留</t>
+  </si>
+  <si>
+    <t>PushMap Intro dwell seconds at each author WP</t>
+  </si>
+  <si>
+    <t>PushMap开战镜头预览在每个作者路点（含起终点）的停留秒数</t>
+  </si>
+  <si>
+    <t>DigTriggerDwellSeconds</t>
+  </si>
+  <si>
+    <t>挖坟触发停留</t>
+  </si>
+  <si>
+    <t>Cursor dwell before DigAction starts</t>
+  </si>
+  <si>
+    <t>光标与可挖坟相交并停留达到本秒数后触发DigAction</t>
+  </si>
+  <si>
+    <t>BaseDigDuration</t>
+  </si>
+  <si>
+    <t>挖坟基础时长</t>
+  </si>
+  <si>
+    <t>BaseDigDuration seconds</t>
+  </si>
+  <si>
+    <t>DigActionDuration=max(下限</t>
+  </si>
+  <si>
+    <t>DigActionDurationFloor</t>
+  </si>
+  <si>
+    <t>挖坟最短时长</t>
+  </si>
+  <si>
+    <t>Min DigActionDuration seconds</t>
+  </si>
+  <si>
+    <t>单次挖坟最短秒数（公式地板）</t>
+  </si>
+  <si>
+    <t>AttackSlotMeleeCount</t>
+  </si>
+  <si>
+    <t>近战攻击位数量</t>
+  </si>
+  <si>
+    <t>Melee AttackSlot ring slot count</t>
+  </si>
+  <si>
+    <t>近战单位围绕目标可占用的攻击位数量</t>
+  </si>
+  <si>
+    <t>AttackSlotRangedCount</t>
+  </si>
+  <si>
+    <t>远程攻击位数量</t>
+  </si>
+  <si>
+    <t>Ranged AttackSlot ring slot count</t>
+  </si>
+  <si>
+    <t>远程单位围绕目标可占用的攻击位数量</t>
+  </si>
+  <si>
+    <t>AttackSlotMargin</t>
+  </si>
+  <si>
+    <t>攻击位环半径余量</t>
+  </si>
+  <si>
+    <t>Ring radius = reach sum - margin</t>
+  </si>
+  <si>
+    <t>攻击位环半径计算时从可达距离减去的余量</t>
+  </si>
+  <si>
+    <t>AttackSlotMinRingRadius</t>
+  </si>
+  <si>
+    <t>攻击位环最小半径</t>
+  </si>
+  <si>
+    <t>Min AttackSlot ring radius</t>
+  </si>
+  <si>
+    <t>攻击位环半径下限</t>
+  </si>
+  <si>
+    <t>AttackSlotReclaimMoveThreshold</t>
+  </si>
+  <si>
+    <t>攻击位重算位移阈值</t>
+  </si>
+  <si>
+    <t>Target move distance to recompute slots</t>
+  </si>
+  <si>
+    <t>目标移动超过本距离时重算攻击位</t>
+  </si>
+  <si>
+    <t>AttackSlotDefaultTargetBodyRadius</t>
+  </si>
+  <si>
+    <t>默认目标体半径</t>
+  </si>
+  <si>
+    <t>Fallback target BodyRadius</t>
+  </si>
+  <si>
+    <t>缺体外观/怪物半径时的默认目标体半径</t>
+  </si>
+  <si>
+    <t>HitConfirmSlack</t>
+  </si>
+  <si>
+    <t>命中确认松弛距离</t>
+  </si>
+  <si>
+    <t>HitConfirm range slack</t>
+  </si>
+  <si>
+    <t>前摇结束命中确认时在攻击距离上额外允许的松弛</t>
+  </si>
+  <si>
+    <t>SurroundGapDegrees</t>
+  </si>
+  <si>
+    <t>包围缺口角度</t>
+  </si>
+  <si>
+    <t>Surround gap sector degrees</t>
+  </si>
+  <si>
+    <t>近战多打一时攻击位环上预留的缺口扇区角度</t>
+  </si>
+  <si>
+    <t>StuckDetectWindowSeconds</t>
+  </si>
+  <si>
+    <t>卡死检测窗口</t>
+  </si>
+  <si>
+    <t>StuckHold detect window seconds</t>
+  </si>
+  <si>
+    <t>有移动意图但位移不足时的检测窗口秒数</t>
+  </si>
+  <si>
+    <t>StuckDisplacementEpsilon</t>
+  </si>
+  <si>
+    <t>卡死位移阈值</t>
+  </si>
+  <si>
+    <t>StuckHold displacement epsilon</t>
+  </si>
+  <si>
+    <t>检测窗口内XZ位移小于本值则判定卡住</t>
+  </si>
+  <si>
+    <t>StuckHoldSeconds</t>
+  </si>
+  <si>
+    <t>卡死停顿时长</t>
+  </si>
+  <si>
+    <t>StuckHold force-Idle seconds</t>
+  </si>
+  <si>
+    <t>判定卡住后强制Idle的秒数</t>
+  </si>
+  <si>
+    <t>ProjectileDefaultHitRadius</t>
+  </si>
+  <si>
+    <t>投射物默认命中半径</t>
+  </si>
+  <si>
+    <t>Default projectile soft-hit radius</t>
+  </si>
+  <si>
+    <t>远程投射物默认软命中半径（表缺列时兜底）</t>
+  </si>
+  <si>
+    <t>DefendVictoryStageExp</t>
+  </si>
+  <si>
+    <t>防守胜利阶段经验</t>
+  </si>
+  <si>
+    <t>Defend victory Demo stage Exp</t>
+  </si>
+  <si>
+    <t>Defend清场胜利结算时入账的阶段经验</t>
+  </si>
+  <si>
+    <t>FlowFieldDefaultCellSize</t>
+  </si>
+  <si>
+    <t>流场默认格宽</t>
+  </si>
+  <si>
+    <t>FlowField default cell size</t>
+  </si>
+  <si>
+    <t>共享目标流场默认格子边长</t>
+  </si>
+  <si>
+    <t>FlowFieldMinCellSize</t>
+  </si>
+  <si>
+    <t>流场最小格宽</t>
+  </si>
+  <si>
+    <t>FlowField min cell size</t>
+  </si>
+  <si>
+    <t>流场格宽下限（性能降级时可抬高）</t>
+  </si>
+  <si>
+    <t>FlowFieldMaxCellSize</t>
+  </si>
+  <si>
+    <t>流场最大格宽</t>
+  </si>
+  <si>
+    <t>FlowField max cell size</t>
+  </si>
+  <si>
+    <t>流场格宽上限</t>
+  </si>
+  <si>
+    <t>MassMoveMaxRecalcPerFrame</t>
+  </si>
+  <si>
+    <t>群体移动每帧重算上限</t>
+  </si>
+  <si>
+    <t>MassMove/AttackSlot refresh budget per frame</t>
+  </si>
+  <si>
+    <t>每帧最多重算路径/攻击位的单位数</t>
+  </si>
+  <si>
+    <t>MassMoveDefaultAgentRadius</t>
+  </si>
+  <si>
+    <t>群体移动默认体半径</t>
+  </si>
+  <si>
+    <t>Default mass-move agent radius</t>
+  </si>
+  <si>
+    <t>群体移动登记时的默认体半径</t>
+  </si>
+  <si>
+    <t>MassMoveArriveEpsilon</t>
+  </si>
+  <si>
+    <t>群体移动到达阈值</t>
+  </si>
+  <si>
+    <t>Arrive epsilon for DesiredDestination</t>
+  </si>
+  <si>
+    <t>到达期望点判定的距离阈值</t>
+  </si>
+  <si>
+    <t>MassMoveDefaultObjectiveArriveRadius</t>
+  </si>
+  <si>
+    <t>目标到达默认半径</t>
+  </si>
+  <si>
+    <t>Default Objective arrive radius</t>
+  </si>
+  <si>
+    <t>目标点到达半径默认值（可被CaptureZone覆盖）</t>
+  </si>
+  <si>
+    <t>MassMoveAttackSlotSeparationScale</t>
+  </si>
+  <si>
+    <t>攻击位软分离系数</t>
+  </si>
+  <si>
+    <t>LocalDetour separation scale in AttackSlot</t>
+  </si>
+  <si>
+    <t>处于攻击位气泡时LocalDetour软分离缩放</t>
+  </si>
+  <si>
+    <t>SoftCollisionMaxCorrectionSpeed</t>
+  </si>
+  <si>
+    <t>软碰撞最大修正速度</t>
+  </si>
+  <si>
+    <t>Soft collision max correction speed</t>
+  </si>
+  <si>
+    <t>软碰撞位置修正速度上限（单位/秒）</t>
+  </si>
+  <si>
+    <t>LocalDetourProbeLength</t>
+  </si>
+  <si>
+    <t>本地绕行探测长度</t>
+  </si>
+  <si>
+    <t>LocalDetour L/R probe length</t>
+  </si>
+  <si>
+    <t>左右绕行探测射线长度</t>
+  </si>
+  <si>
+    <t>LocalDetourSoftSeparationStrength</t>
+  </si>
+  <si>
+    <t>本地绕行软分离强度</t>
+  </si>
+  <si>
+    <t>LocalDetour soft separation strength</t>
+  </si>
+  <si>
+    <t>友军软分离推力强度</t>
+  </si>
+  <si>
+    <t>LocalDetourDetourBias</t>
+  </si>
+  <si>
+    <t>本地绕行偏置</t>
+  </si>
+  <si>
+    <t>LocalDetour L/R bias blend</t>
+  </si>
+  <si>
+    <t>绕行方向与原期望方向的混合偏置</t>
+  </si>
+  <si>
+    <t>LocalDetourForwardConeHalfAngleDeg</t>
+  </si>
+  <si>
+    <t>本地绕行前向锥半角</t>
+  </si>
+  <si>
+    <t>Forward block cone half-angle degrees</t>
+  </si>
+  <si>
+    <t>判定前方友军阻挡的圆锥半角（度）</t>
+  </si>
+  <si>
+    <t>BossAdvanceArriveRadius</t>
+  </si>
+  <si>
+    <t>Boss推进到达半径</t>
+  </si>
+  <si>
+    <t>BossPoint advance arrive radius</t>
+  </si>
+  <si>
+    <t>目标链耗尽后推进Boss点的到达半径</t>
+  </si>
+  <si>
+    <t>EngageStickHysteresisMargin</t>
+  </si>
+  <si>
+    <t>接战粘滞余量</t>
+  </si>
+  <si>
+    <t>Engage sticky retarget hysteresis</t>
+  </si>
+  <si>
+    <t>接战粘滞：新目标需更近超过本余量才换目标</t>
+  </si>
+  <si>
+    <t>PushMapSpawnMinSampleDistance</t>
+  </si>
+  <si>
+    <t>刷怪散布最小采样距</t>
+  </si>
+  <si>
+    <t>PushMap spawn min sample distance</t>
+  </si>
+  <si>
+    <t>刷怪散布环形采样的最小间距</t>
+  </si>
+  <si>
+    <t>PushMapSpawnSampleDistanceBodyMul</t>
+  </si>
+  <si>
+    <t>刷怪散布体半径倍数</t>
+  </si>
+  <si>
+    <t>Spawn sample distance = max(min</t>
+  </si>
+  <si>
+    <t>r*mul)</t>
+  </si>
+  <si>
+    <t>PushMapSpawnLeashSlack</t>
+  </si>
+  <si>
+    <t>刷怪拴绳松弛</t>
+  </si>
+  <si>
+    <t>NavMesh sample leash slack</t>
+  </si>
+  <si>
+    <t>刷怪SamplePosition相对基点的拴绳松弛</t>
+  </si>
+  <si>
+    <t>PushMapSpawnAbsoluteLeashFloor</t>
+  </si>
+  <si>
+    <t>刷怪绝对拴绳下限</t>
+  </si>
+  <si>
+    <t>Absolute leash floor</t>
+  </si>
+  <si>
+    <t>刷怪绝对拴绳距离下限</t>
+  </si>
+  <si>
+    <t>PushMapSpawnAbsoluteLeashBodyMul</t>
+  </si>
+  <si>
+    <t>刷怪绝对拴绳体倍数</t>
+  </si>
+  <si>
+    <t>Absolute leash = max(floor</t>
+  </si>
+  <si>
+    <t>r*mul)</t>
   </si>
 </sst>
 </file>
@@ -538,62 +1126,62 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{152188F9-B4F1-4AA8-8C2D-95D7862DEBAB}">
-  <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E58"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
         <v>6</v>
-      </c>
-      <c r="D1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
       </c>
       <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
       </c>
       <c r="E3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -610,7 +1198,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -627,7 +1215,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -644,7 +1232,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -661,7 +1249,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -678,7 +1266,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -695,8 +1283,839 @@
         <v>38</v>
       </c>
     </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10">
+        <v>18</v>
+      </c>
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11">
+        <v>1.5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13">
+        <v>0.1</v>
+      </c>
+      <c r="D13" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14">
+        <v>100</v>
+      </c>
+      <c r="D14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15">
+        <v>0.15</v>
+      </c>
+      <c r="D15" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16">
+        <v>0.25</v>
+      </c>
+      <c r="D16" t="s">
+        <v>65</v>
+      </c>
+      <c r="E16" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17">
+        <v>0.5</v>
+      </c>
+      <c r="D17" t="s">
+        <v>69</v>
+      </c>
+      <c r="E17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18">
+        <v>0.5</v>
+      </c>
+      <c r="D18" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19">
+        <v>20</v>
+      </c>
+      <c r="D19" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20">
+        <v>4</v>
+      </c>
+      <c r="D20" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" t="s">
+        <v>84</v>
+      </c>
+      <c r="C21">
+        <v>1.5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>85</v>
+      </c>
+      <c r="E21" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>87</v>
+      </c>
+      <c r="B22" t="s">
+        <v>88</v>
+      </c>
+      <c r="C22">
+        <v>0.5</v>
+      </c>
+      <c r="D22" t="s">
+        <v>89</v>
+      </c>
+      <c r="E22" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>91</v>
+      </c>
+      <c r="B23" t="s">
+        <v>92</v>
+      </c>
+      <c r="C23">
+        <v>0.2</v>
+      </c>
+      <c r="D23" t="s">
+        <v>93</v>
+      </c>
+      <c r="E23" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>95</v>
+      </c>
+      <c r="B24" t="s">
+        <v>96</v>
+      </c>
+      <c r="C24">
+        <v>0.8</v>
+      </c>
+      <c r="D24" t="s">
+        <v>97</v>
+      </c>
+      <c r="E24" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" t="s">
+        <v>100</v>
+      </c>
+      <c r="C25">
+        <v>0.1</v>
+      </c>
+      <c r="D25" t="s">
+        <v>101</v>
+      </c>
+      <c r="E25" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>103</v>
+      </c>
+      <c r="B26" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26">
+        <v>12</v>
+      </c>
+      <c r="D26" t="s">
+        <v>105</v>
+      </c>
+      <c r="E26" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" t="s">
+        <v>107</v>
+      </c>
+      <c r="B27" t="s">
+        <v>108</v>
+      </c>
+      <c r="C27">
+        <v>8</v>
+      </c>
+      <c r="D27" t="s">
+        <v>109</v>
+      </c>
+      <c r="E27" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" t="s">
+        <v>111</v>
+      </c>
+      <c r="B28" t="s">
+        <v>112</v>
+      </c>
+      <c r="C28">
+        <v>0.05</v>
+      </c>
+      <c r="D28" t="s">
+        <v>113</v>
+      </c>
+      <c r="E28" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" t="s">
+        <v>115</v>
+      </c>
+      <c r="B29" t="s">
+        <v>116</v>
+      </c>
+      <c r="C29">
+        <v>0.05</v>
+      </c>
+      <c r="D29" t="s">
+        <v>117</v>
+      </c>
+      <c r="E29" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" t="s">
+        <v>119</v>
+      </c>
+      <c r="B30" t="s">
+        <v>120</v>
+      </c>
+      <c r="C30">
+        <v>0.5</v>
+      </c>
+      <c r="D30" t="s">
+        <v>121</v>
+      </c>
+      <c r="E30" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" t="s">
+        <v>123</v>
+      </c>
+      <c r="B31" t="s">
+        <v>124</v>
+      </c>
+      <c r="C31">
+        <v>0.35</v>
+      </c>
+      <c r="D31" t="s">
+        <v>125</v>
+      </c>
+      <c r="E31" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" t="s">
+        <v>127</v>
+      </c>
+      <c r="B32" t="s">
+        <v>128</v>
+      </c>
+      <c r="C32">
+        <v>0.05</v>
+      </c>
+      <c r="D32" t="s">
+        <v>129</v>
+      </c>
+      <c r="E32" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" t="s">
+        <v>131</v>
+      </c>
+      <c r="B33" t="s">
+        <v>132</v>
+      </c>
+      <c r="C33">
+        <v>60</v>
+      </c>
+      <c r="D33" t="s">
+        <v>133</v>
+      </c>
+      <c r="E33" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" t="s">
+        <v>135</v>
+      </c>
+      <c r="B34" t="s">
+        <v>136</v>
+      </c>
+      <c r="C34">
+        <v>0.5</v>
+      </c>
+      <c r="D34" t="s">
+        <v>137</v>
+      </c>
+      <c r="E34" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" t="s">
+        <v>139</v>
+      </c>
+      <c r="B35" t="s">
+        <v>140</v>
+      </c>
+      <c r="C35">
+        <v>0.2</v>
+      </c>
+      <c r="D35" t="s">
+        <v>141</v>
+      </c>
+      <c r="E35" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" t="s">
+        <v>143</v>
+      </c>
+      <c r="B36" t="s">
+        <v>144</v>
+      </c>
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="D36" t="s">
+        <v>145</v>
+      </c>
+      <c r="E36" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" t="s">
+        <v>147</v>
+      </c>
+      <c r="B37" t="s">
+        <v>148</v>
+      </c>
+      <c r="C37">
+        <v>0.55</v>
+      </c>
+      <c r="D37" t="s">
+        <v>149</v>
+      </c>
+      <c r="E37" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" t="s">
+        <v>151</v>
+      </c>
+      <c r="B38" t="s">
+        <v>152</v>
+      </c>
+      <c r="C38">
+        <v>100</v>
+      </c>
+      <c r="D38" t="s">
+        <v>153</v>
+      </c>
+      <c r="E38" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" t="s">
+        <v>155</v>
+      </c>
+      <c r="B39" t="s">
+        <v>156</v>
+      </c>
+      <c r="C39">
+        <v>0.5</v>
+      </c>
+      <c r="D39" t="s">
+        <v>157</v>
+      </c>
+      <c r="E39" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" t="s">
+        <v>159</v>
+      </c>
+      <c r="B40" t="s">
+        <v>160</v>
+      </c>
+      <c r="C40">
+        <v>0.25</v>
+      </c>
+      <c r="D40" t="s">
+        <v>161</v>
+      </c>
+      <c r="E40" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" t="s">
+        <v>163</v>
+      </c>
+      <c r="B41" t="s">
+        <v>164</v>
+      </c>
+      <c r="C41">
+        <v>0.5</v>
+      </c>
+      <c r="D41" t="s">
+        <v>165</v>
+      </c>
+      <c r="E41" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" t="s">
+        <v>167</v>
+      </c>
+      <c r="B42" t="s">
+        <v>168</v>
+      </c>
+      <c r="C42">
+        <v>50</v>
+      </c>
+      <c r="D42" t="s">
+        <v>169</v>
+      </c>
+      <c r="E42" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" t="s">
+        <v>171</v>
+      </c>
+      <c r="B43" t="s">
+        <v>172</v>
+      </c>
+      <c r="C43">
+        <v>0.1</v>
+      </c>
+      <c r="D43" t="s">
+        <v>173</v>
+      </c>
+      <c r="E43" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" t="s">
+        <v>175</v>
+      </c>
+      <c r="B44" t="s">
+        <v>176</v>
+      </c>
+      <c r="C44">
+        <v>0.08</v>
+      </c>
+      <c r="D44" t="s">
+        <v>177</v>
+      </c>
+      <c r="E44" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" t="s">
+        <v>179</v>
+      </c>
+      <c r="B45" t="s">
+        <v>180</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+      <c r="D45" t="s">
+        <v>181</v>
+      </c>
+      <c r="E45" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" t="s">
+        <v>183</v>
+      </c>
+      <c r="B46" t="s">
+        <v>184</v>
+      </c>
+      <c r="C46">
+        <v>0.35</v>
+      </c>
+      <c r="D46" t="s">
+        <v>185</v>
+      </c>
+      <c r="E46" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" t="s">
+        <v>187</v>
+      </c>
+      <c r="B47" t="s">
+        <v>188</v>
+      </c>
+      <c r="C47">
+        <v>2</v>
+      </c>
+      <c r="D47" t="s">
+        <v>189</v>
+      </c>
+      <c r="E47" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" t="s">
+        <v>191</v>
+      </c>
+      <c r="B48" t="s">
+        <v>192</v>
+      </c>
+      <c r="C48">
+        <v>1</v>
+      </c>
+      <c r="D48" t="s">
+        <v>193</v>
+      </c>
+      <c r="E48" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49" t="s">
+        <v>195</v>
+      </c>
+      <c r="B49" t="s">
+        <v>196</v>
+      </c>
+      <c r="C49">
+        <v>0.15</v>
+      </c>
+      <c r="D49" t="s">
+        <v>197</v>
+      </c>
+      <c r="E49" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50" t="s">
+        <v>199</v>
+      </c>
+      <c r="B50" t="s">
+        <v>200</v>
+      </c>
+      <c r="C50">
+        <v>0.85</v>
+      </c>
+      <c r="D50" t="s">
+        <v>201</v>
+      </c>
+      <c r="E50" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51" t="s">
+        <v>203</v>
+      </c>
+      <c r="B51" t="s">
+        <v>204</v>
+      </c>
+      <c r="C51">
+        <v>50</v>
+      </c>
+      <c r="D51" t="s">
+        <v>205</v>
+      </c>
+      <c r="E51" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52" t="s">
+        <v>207</v>
+      </c>
+      <c r="B52" t="s">
+        <v>208</v>
+      </c>
+      <c r="C52">
+        <v>0.35</v>
+      </c>
+      <c r="D52" t="s">
+        <v>209</v>
+      </c>
+      <c r="E52" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53" t="s">
+        <v>211</v>
+      </c>
+      <c r="B53" t="s">
+        <v>212</v>
+      </c>
+      <c r="C53">
+        <v>0.15</v>
+      </c>
+      <c r="D53" t="s">
+        <v>213</v>
+      </c>
+      <c r="E53" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54" t="s">
+        <v>215</v>
+      </c>
+      <c r="B54" t="s">
+        <v>216</v>
+      </c>
+      <c r="C54">
+        <v>0.75</v>
+      </c>
+      <c r="D54" t="s">
+        <v>217</v>
+      </c>
+      <c r="E54" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55" t="s">
+        <v>219</v>
+      </c>
+      <c r="B55" t="s">
+        <v>220</v>
+      </c>
+      <c r="C55">
+        <v>2.5</v>
+      </c>
+      <c r="D55" t="s">
+        <v>221</v>
+      </c>
+      <c r="E55" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56" t="s">
+        <v>223</v>
+      </c>
+      <c r="B56" t="s">
+        <v>224</v>
+      </c>
+      <c r="C56">
+        <v>0.35</v>
+      </c>
+      <c r="D56" t="s">
+        <v>225</v>
+      </c>
+      <c r="E56" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" t="s">
+        <v>227</v>
+      </c>
+      <c r="B57" t="s">
+        <v>228</v>
+      </c>
+      <c r="C57">
+        <v>3</v>
+      </c>
+      <c r="D57" t="s">
+        <v>229</v>
+      </c>
+      <c r="E57" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" t="s">
+        <v>231</v>
+      </c>
+      <c r="B58" t="s">
+        <v>232</v>
+      </c>
+      <c r="C58">
+        <v>10</v>
+      </c>
+      <c r="D58" t="s">
+        <v>233</v>
+      </c>
+      <c r="E58" t="s">
+        <v>234</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>